<commit_message>
Tweaking zero reviews to not take this year
Hail Mary clause
</commit_message>
<xml_diff>
--- a/Official Whitelist.xlsx
+++ b/Official Whitelist.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bigba\aa Personal Projects\Letterboxd-List-Scraping\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E020EF68-3684-42A3-BD5D-4C59ABB3A091}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8CB09E4E-20A8-4260-8B6D-DEBD217B0567}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="711" uniqueCount="711">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="751" uniqueCount="751">
   <si>
     <t>Title</t>
   </si>
@@ -2158,6 +2158,126 @@
   </si>
   <si>
     <t>https://letterboxd.com/film/the-wolf-house/</t>
+  </si>
+  <si>
+    <t>The Ox Bow Incident</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/the-ox-bow-incident/</t>
+  </si>
+  <si>
+    <t>Mustang</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/mustang-2015/</t>
+  </si>
+  <si>
+    <t>Fargo</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/fargo/</t>
+  </si>
+  <si>
+    <t>Punishment Park</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/punishment-park/</t>
+  </si>
+  <si>
+    <t>The Gold Rush</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/the-gold-rush/</t>
+  </si>
+  <si>
+    <t>Mulan</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/mulan/</t>
+  </si>
+  <si>
+    <t>Il Posto</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/il-posto/</t>
+  </si>
+  <si>
+    <t>Dead Mans Letters</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/dead-mans-letters/</t>
+  </si>
+  <si>
+    <t>Sanjuro</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/sanjuro/</t>
+  </si>
+  <si>
+    <t>Monty Python And The Holy Grail</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/monty-python-and-the-holy-grail/</t>
+  </si>
+  <si>
+    <t>Pink Floyd The Wall</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/pink-floyd-the-wall/</t>
+  </si>
+  <si>
+    <t>The Umbrellas Of Cherbourg</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/the-umbrellas-of-cherbourg/</t>
+  </si>
+  <si>
+    <t>Crayon Shin Chan The Adult Empire Strikes</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/crayon-shin-chan-the-adult-empire-strikes/</t>
+  </si>
+  <si>
+    <t>Reservoir Dogs</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/reservoir-dogs/</t>
+  </si>
+  <si>
+    <t>Rope</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/rope/</t>
+  </si>
+  <si>
+    <t>Souleymane's Story</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/souleymanes-story/</t>
+  </si>
+  <si>
+    <t>Ballad of a Soldier</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/ballad-of-a-soldier/</t>
+  </si>
+  <si>
+    <t>Happiness 1965</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/happiness-1965/</t>
+  </si>
+  <si>
+    <t>The Color of Pomegranates</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/the-color-of-pomegranates/</t>
+  </si>
+  <si>
+    <t>Rap World</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/rap-world/</t>
   </si>
 </sst>
 </file>
@@ -2498,7 +2618,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D355"/>
+  <dimension ref="A1:D375"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="46.36328125" bestFit="1" customWidth="1"/>
@@ -6415,6 +6535,226 @@
         <v>710</v>
       </c>
     </row>
+    <row r="356" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A356" t="s">
+        <v>711</v>
+      </c>
+      <c r="B356">
+        <v>1943</v>
+      </c>
+      <c r="D356" t="s">
+        <v>712</v>
+      </c>
+    </row>
+    <row r="357" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A357" t="s">
+        <v>713</v>
+      </c>
+      <c r="B357">
+        <v>2015</v>
+      </c>
+      <c r="D357" t="s">
+        <v>714</v>
+      </c>
+    </row>
+    <row r="358" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A358" t="s">
+        <v>715</v>
+      </c>
+      <c r="B358">
+        <v>1996</v>
+      </c>
+      <c r="D358" t="s">
+        <v>716</v>
+      </c>
+    </row>
+    <row r="359" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A359" t="s">
+        <v>717</v>
+      </c>
+      <c r="B359">
+        <v>1971</v>
+      </c>
+      <c r="D359" t="s">
+        <v>718</v>
+      </c>
+    </row>
+    <row r="360" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A360" t="s">
+        <v>719</v>
+      </c>
+      <c r="B360">
+        <v>1925</v>
+      </c>
+      <c r="D360" t="s">
+        <v>720</v>
+      </c>
+    </row>
+    <row r="361" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A361" t="s">
+        <v>721</v>
+      </c>
+      <c r="B361">
+        <v>1998</v>
+      </c>
+      <c r="D361" t="s">
+        <v>722</v>
+      </c>
+    </row>
+    <row r="362" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A362" t="s">
+        <v>723</v>
+      </c>
+      <c r="B362">
+        <v>1961</v>
+      </c>
+      <c r="D362" t="s">
+        <v>724</v>
+      </c>
+    </row>
+    <row r="363" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A363" t="s">
+        <v>725</v>
+      </c>
+      <c r="B363">
+        <v>1986</v>
+      </c>
+      <c r="D363" t="s">
+        <v>726</v>
+      </c>
+    </row>
+    <row r="364" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A364" t="s">
+        <v>727</v>
+      </c>
+      <c r="B364">
+        <v>1962</v>
+      </c>
+      <c r="D364" t="s">
+        <v>728</v>
+      </c>
+    </row>
+    <row r="365" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A365" t="s">
+        <v>729</v>
+      </c>
+      <c r="B365">
+        <v>1975</v>
+      </c>
+      <c r="D365" t="s">
+        <v>730</v>
+      </c>
+    </row>
+    <row r="366" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A366" t="s">
+        <v>731</v>
+      </c>
+      <c r="B366">
+        <v>1982</v>
+      </c>
+      <c r="D366" t="s">
+        <v>732</v>
+      </c>
+    </row>
+    <row r="367" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A367" t="s">
+        <v>733</v>
+      </c>
+      <c r="B367">
+        <v>1964</v>
+      </c>
+      <c r="D367" t="s">
+        <v>734</v>
+      </c>
+    </row>
+    <row r="368" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A368" t="s">
+        <v>735</v>
+      </c>
+      <c r="B368">
+        <v>2001</v>
+      </c>
+      <c r="D368" t="s">
+        <v>736</v>
+      </c>
+    </row>
+    <row r="369" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A369" t="s">
+        <v>737</v>
+      </c>
+      <c r="B369">
+        <v>1992</v>
+      </c>
+      <c r="D369" t="s">
+        <v>738</v>
+      </c>
+    </row>
+    <row r="370" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A370" t="s">
+        <v>739</v>
+      </c>
+      <c r="B370">
+        <v>1948</v>
+      </c>
+      <c r="D370" t="s">
+        <v>740</v>
+      </c>
+    </row>
+    <row r="371" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A371" t="s">
+        <v>741</v>
+      </c>
+      <c r="B371">
+        <v>2024</v>
+      </c>
+      <c r="D371" t="s">
+        <v>742</v>
+      </c>
+    </row>
+    <row r="372" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A372" t="s">
+        <v>743</v>
+      </c>
+      <c r="B372">
+        <v>1959</v>
+      </c>
+      <c r="D372" t="s">
+        <v>744</v>
+      </c>
+    </row>
+    <row r="373" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A373" t="s">
+        <v>745</v>
+      </c>
+      <c r="B373">
+        <v>1965</v>
+      </c>
+      <c r="D373" t="s">
+        <v>746</v>
+      </c>
+    </row>
+    <row r="374" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A374" t="s">
+        <v>747</v>
+      </c>
+      <c r="B374">
+        <v>1969</v>
+      </c>
+      <c r="D374" t="s">
+        <v>748</v>
+      </c>
+    </row>
+    <row r="375" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A375" t="s">
+        <v>749</v>
+      </c>
+      <c r="B375">
+        <v>2024</v>
+      </c>
+      <c r="D375" t="s">
+        <v>750</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Updating so that new movies are added to zero_reviews
</commit_message>
<xml_diff>
--- a/Official Whitelist.xlsx
+++ b/Official Whitelist.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bigba\aa Personal Projects\Letterboxd-List-Scraping\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8CB09E4E-20A8-4260-8B6D-DEBD217B0567}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A9F3783-45F1-476F-9FFE-ACA917C05B74}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="751" uniqueCount="751">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1055" uniqueCount="1054">
   <si>
     <t>Title</t>
   </si>
@@ -2278,13 +2278,922 @@
   </si>
   <si>
     <t>https://letterboxd.com/film/rap-world/</t>
+  </si>
+  <si>
+    <t>Center Stage</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/center-stage-1991/</t>
+  </si>
+  <si>
+    <t>Kandukondain Kandukondain</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/kandukondain-kandukondain/</t>
+  </si>
+  <si>
+    <t>An Angel At My Table</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/an-angel-at-my-table/</t>
+  </si>
+  <si>
+    <t>Gone With The Wind</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/gone-with-the-wind/</t>
+  </si>
+  <si>
+    <t>Topsy Turvy</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/topsy-turvy/</t>
+  </si>
+  <si>
+    <t>Barfi</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/barfi/</t>
+  </si>
+  <si>
+    <t>Empire Of The Sun</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/empire-of-the-sun/</t>
+  </si>
+  <si>
+    <t>West Side Story</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/west-side-story/</t>
+  </si>
+  <si>
+    <t>How To Train Your Dragon</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/how-to-train-your-dragon/</t>
+  </si>
+  <si>
+    <t>Phantom Of The Paradise</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/phantom-of-the-paradise/</t>
+  </si>
+  <si>
+    <t>Street Of Shame</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/street-of-shame/</t>
+  </si>
+  <si>
+    <t>Kaguya Sama Love Is War The First Kiss That Never Ends</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/kaguya-sama-love-is-war-the-first-kiss-that-never-ends/</t>
+  </si>
+  <si>
+    <t>Project Hail Mary</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/project-hail-mary/</t>
+  </si>
+  <si>
+    <t>The Cameraman</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/the-cameraman/</t>
+  </si>
+  <si>
+    <t>A Short Film About Killing</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/a-short-film-about-killing/</t>
+  </si>
+  <si>
+    <t>Sonatine</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/sonatine/</t>
+  </si>
+  <si>
+    <t>After Hours</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/after-hours/</t>
+  </si>
+  <si>
+    <t>Beau Travail</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/beau-travail/</t>
+  </si>
+  <si>
+    <t>Kanal 1957</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/kanal-1957/</t>
+  </si>
+  <si>
+    <t>Shrek</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/shrek/</t>
+  </si>
+  <si>
+    <t>The Innocents</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/the-innocents/</t>
+  </si>
+  <si>
+    <t>Ponyo</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/ponyo/</t>
+  </si>
+  <si>
+    <t>What We Do In The Shadows</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/what-we-do-in-the-shadows/</t>
+  </si>
+  <si>
+    <t>Trouble In Paradise</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/trouble-in-paradise/</t>
+  </si>
+  <si>
+    <t>Shrek 2</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/shrek-2/</t>
+  </si>
+  <si>
+    <t>Monicas Gang In An Adventure In Time</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/monicas-gang-in-an-adventure-in-time/</t>
+  </si>
+  <si>
+    <t>Safety Last</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/safety-last/</t>
+  </si>
+  <si>
+    <t>Harold And Maude</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/harold-and-maude/</t>
+  </si>
+  <si>
+    <t>Whats Up Doc 1972</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/whats-up-doc-1972/</t>
+  </si>
+  <si>
+    <t>A Short Film About Love</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/a-short-film-about-love/</t>
+  </si>
+  <si>
+    <t>Women On The Verge Of A Nervous Breakdown</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/women-on-the-verge-of-a-nervous-breakdown/</t>
+  </si>
+  <si>
+    <t>Toy Story</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/toy-story/</t>
+  </si>
+  <si>
+    <t>Out Of The Past</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/out-of-the-past/</t>
+  </si>
+  <si>
+    <t>My Darling Clementine</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/my-darling-clementine/</t>
+  </si>
+  <si>
+    <t>Lady Snowblood</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/lady-snowblood/</t>
+  </si>
+  <si>
+    <t>Aguirre The Wrath Of God</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/aguirre-the-wrath-of-god/</t>
+  </si>
+  <si>
+    <t>I Am a Fugitive from a Chain Gang</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/i-am-a-fugitive-from-a-chain-gang/</t>
+  </si>
+  <si>
+    <t>The Big Heat</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/the-big-heat/</t>
+  </si>
+  <si>
+    <t>3 Iron</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/3-iron/</t>
+  </si>
+  <si>
+    <t>Last Year At Marienbad</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/last-year-at-marienbad/</t>
+  </si>
+  <si>
+    <t>The Double Life of VÃ©ronique</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/the-double-life-of-veronique/</t>
+  </si>
+  <si>
+    <t>Up</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/up/</t>
+  </si>
+  <si>
+    <t>Tangerines</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/tangerines/</t>
+  </si>
+  <si>
+    <t>His Motorbike, Her Island</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/his-motorbike-her-island/</t>
+  </si>
+  <si>
+    <t>Petite Maman</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/petite-maman/</t>
+  </si>
+  <si>
+    <t>Elevator To The Gallows</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/elevator-to-the-gallows/</t>
+  </si>
+  <si>
+    <t>The Princess Bride</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/the-princess-bride/</t>
+  </si>
+  <si>
+    <t>Paprika 2006</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/paprika-2006/</t>
+  </si>
+  <si>
+    <t>Angels Egg</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/angels-egg/</t>
+  </si>
+  <si>
+    <t>Viridiana</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/viridiana/</t>
+  </si>
+  <si>
+    <t>Days Of Heaven</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/days-of-heaven/</t>
+  </si>
+  <si>
+    <t>Oslo, August 31st</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/oslo-august-31st/</t>
+  </si>
+  <si>
+    <t>Dou Kyu Sei Classmates</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/dou-kyu-sei-classmates/</t>
+  </si>
+  <si>
+    <t>Ghost In The Shell</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/ghost-in-the-shell/</t>
+  </si>
+  <si>
+    <t>The Crowd</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/the-crowd/</t>
+  </si>
+  <si>
+    <t>The Quiet Girl</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/the-quiet-girl/</t>
+  </si>
+  <si>
+    <t>The Breadwinner</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/the-breadwinner/</t>
+  </si>
+  <si>
+    <t>Whos Singin Over There</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/whos-singin-over-there/</t>
+  </si>
+  <si>
+    <t>Flow 2024</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/flow-2024/</t>
+  </si>
+  <si>
+    <t>Letter From An Unknown Woman</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/letter-from-an-unknown-woman/</t>
+  </si>
+  <si>
+    <t>Sidewalls</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/sidewalls/</t>
+  </si>
+  <si>
+    <t>Forbidden Games 1952</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/forbidden-games-1952/</t>
+  </si>
+  <si>
+    <t>Little Amelie Or The Character Of Rain</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/little-amelie-or-the-character-of-rain/</t>
+  </si>
+  <si>
+    <t>Orpheus</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/orpheus/</t>
+  </si>
+  <si>
+    <t>Black Girl</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/black-girl-1966/</t>
+  </si>
+  <si>
+    <t>Nothing But A Man</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/nothing-but-a-man/</t>
+  </si>
+  <si>
+    <t>Beauty And The Beast</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/beauty-and-the-beast/</t>
+  </si>
+  <si>
+    <t>Blindspotting</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/blindspotting/</t>
+  </si>
+  <si>
+    <t>Letter Never Sent</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/letter-never-sent/</t>
+  </si>
+  <si>
+    <t>Monsters Inc</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/monsters-inc/</t>
+  </si>
+  <si>
+    <t>Au Hasard Balthazar</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/au-hasard-balthazar/</t>
+  </si>
+  <si>
+    <t>True Stories</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/true-stories/</t>
+  </si>
+  <si>
+    <t>The War Game</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/the-war-game/</t>
+  </si>
+  <si>
+    <t>Hedwig And The Angry Inch</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/hedwig-and-the-angry-inch/</t>
+  </si>
+  <si>
+    <t>Ratcatcher</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/ratcatcher/</t>
+  </si>
+  <si>
+    <t>Three Men And A Leg</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/three-men-and-a-leg/</t>
+  </si>
+  <si>
+    <t>The Prince Of Egypt</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/the-prince-of-egypt/</t>
+  </si>
+  <si>
+    <t>Eternity</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/eternity-2017/</t>
+  </si>
+  <si>
+    <t>Shoeshine</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/shoeshine/</t>
+  </si>
+  <si>
+    <t>One Piece Baron Omatsuri And The Secret Island</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/one-piece-baron-omatsuri-and-the-secret-island/</t>
+  </si>
+  <si>
+    <t>The Music Room</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/the-music-room/</t>
+  </si>
+  <si>
+    <t>Kuroneko</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/kuroneko/</t>
+  </si>
+  <si>
+    <t>The Summit Of The Gods</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/the-summit-of-the-gods/</t>
+  </si>
+  <si>
+    <t>Given The Movie To The Sea</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/given-the-movie-to-the-sea/</t>
+  </si>
+  <si>
+    <t>All That Heaven Allows</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/all-that-heaven-allows/</t>
+  </si>
+  <si>
+    <t>When Harry Met Sally</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/when-harry-met-sally/</t>
+  </si>
+  <si>
+    <t>Songs From The Second Floor</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/songs-from-the-second-floor/</t>
+  </si>
+  <si>
+    <t>The Circus</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/the-circus/</t>
+  </si>
+  <si>
+    <t>Lilo Stitch</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/lilo-stitch/</t>
+  </si>
+  <si>
+    <t>Shadows of Forgotten Ancestors</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/shadows-of-forgotten-ancestors/</t>
+  </si>
+  <si>
+    <t>Boy</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/boy-2010/</t>
+  </si>
+  <si>
+    <t>Kizumonogatari Part 2: Nekketsu</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/kizumonogatari-part-2-nekketsu/</t>
+  </si>
+  <si>
+    <t>The Cabinet Of Dr Caligari 1920</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/the-cabinet-of-dr-caligari-1920/</t>
+  </si>
+  <si>
+    <t>The Muppet Christmas Carol</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/the-muppet-christmas-carol/</t>
+  </si>
+  <si>
+    <t>The Watermelon Woman</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/the-watermelon-woman/</t>
+  </si>
+  <si>
+    <t>Godzilla</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/godzilla/</t>
+  </si>
+  <si>
+    <t>The Farewell 2019</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/the-farewell-2019/</t>
+  </si>
+  <si>
+    <t>The Fabulous Baron Munchausen</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/the-fabulous-baron-munchausen/</t>
+  </si>
+  <si>
+    <t>One Cut Of The Dead</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/one-cut-of-the-dead/</t>
+  </si>
+  <si>
+    <t>Mouchette</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/mouchette/</t>
+  </si>
+  <si>
+    <t>10 Things I Hate About You</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/10-things-i-hate-about-you/</t>
+  </si>
+  <si>
+    <t>The Muppet Movie</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/the-muppet-movie/</t>
+  </si>
+  <si>
+    <t>The Wind</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/the-wind/</t>
+  </si>
+  <si>
+    <t>Kisapmata</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/kisapmata/</t>
+  </si>
+  <si>
+    <t>The Last Laugh</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/the-last-laugh/</t>
+  </si>
+  <si>
+    <t>Cold War 2018</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/cold-war-2018/</t>
+  </si>
+  <si>
+    <t>The Rocky Horror Picture Show</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/the-rocky-horror-picture-show/</t>
+  </si>
+  <si>
+    <t>Mononoke The Movie Chapter Ii The Ashes Of</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/mononoke-the-movie-chapter-ii-the-ashes-of/</t>
+  </si>
+  <si>
+    <t>Batman Mask Of The Phantasm</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/batman-mask-of-the-phantasm/</t>
+  </si>
+  <si>
+    <t>Four Adventures Of Reinette And Mirabelle</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/four-adventures-of-reinette-and-mirabelle/</t>
+  </si>
+  <si>
+    <t>Ivan the Terrible, Part II: The Boyars' Plot</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/ivan-the-terrible-part-ii-the-boyars-plot/</t>
+  </si>
+  <si>
+    <t>Ida</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/ida/</t>
+  </si>
+  <si>
+    <t>Insiang</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/insiang/</t>
+  </si>
+  <si>
+    <t>Lovers Rock 2020</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/lovers-rock-2020/</t>
+  </si>
+  <si>
+    <t>Laura</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/laura/</t>
+  </si>
+  <si>
+    <t>Young Hearts</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/young-hearts-2024/</t>
+  </si>
+  <si>
+    <t>The King And The Mockingbird</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/the-king-and-the-mockingbird/</t>
+  </si>
+  <si>
+    <t>Devi</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/devi/</t>
+  </si>
+  <si>
+    <t>Pariah</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/pariah/</t>
+  </si>
+  <si>
+    <t>The Swimmer</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/the-swimmer/</t>
+  </si>
+  <si>
+    <t>Day Of The Wacko</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/day-of-the-wacko/</t>
+  </si>
+  <si>
+    <t>I Daniel Blake</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/i-daniel-blake/</t>
+  </si>
+  <si>
+    <t>Tangled</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/tangled-2010/</t>
+  </si>
+  <si>
+    <t>The 8 Diagram Pole Fighter</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/the-8-diagram-pole-fighter/</t>
+  </si>
+  <si>
+    <t>Superstar The Karen Carpenter Story</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/superstar-the-karen-carpenter-story/</t>
+  </si>
+  <si>
+    <t>Night And The City</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/night-and-the-city/</t>
+  </si>
+  <si>
+    <t>U.S. Go Home</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/us-go-home/</t>
+  </si>
+  <si>
+    <t>Farha</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/farha/</t>
+  </si>
+  <si>
+    <t>My Little Pony Equestria Girls Rainbow Rocks</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/my-little-pony-equestria-girls-rainbow-rocks/</t>
+  </si>
+  <si>
+    <t>Buddies</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/buddies-1985/</t>
+  </si>
+  <si>
+    <t>The Boys</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/the-boys/</t>
+  </si>
+  <si>
+    <t>Maronas Fantastic Tale</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/maronas-fantastic-tale/</t>
+  </si>
+  <si>
+    <t>Land Of Mine</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/land-of-mine/</t>
+  </si>
+  <si>
+    <t>Black Dynamite</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/black-dynamite/</t>
+  </si>
+  <si>
+    <t>Frances Ha</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/frances-ha/</t>
+  </si>
+  <si>
+    <t>His Girl Friday</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/his-girl-friday/</t>
+  </si>
+  <si>
+    <t>The Chorus</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/the-chorus/</t>
+  </si>
+  <si>
+    <t>Pale Flower</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/pale-flower/</t>
+  </si>
+  <si>
+    <t>Saving Face</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/saving-face/</t>
+  </si>
+  <si>
+    <t>Sunshine</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/sunshine-2024/</t>
+  </si>
+  <si>
+    <t>Love in the Afternoon</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/love-in-the-afternoon-1972/</t>
+  </si>
+  <si>
+    <t>Porco Rosso</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/porco-rosso/</t>
+  </si>
+  <si>
+    <t>A Town Called Panic</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/a-town-called-panic/</t>
+  </si>
+  <si>
+    <t>Balkan Spy</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/balkan-spy/</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/babylon/</t>
+  </si>
+  <si>
+    <t>Finding Nemo</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/finding-nemo/</t>
+  </si>
+  <si>
+    <t>Hunger</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/hunger/</t>
+  </si>
+  <si>
+    <t>The Triplets Of Belleville</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/the-triplets-of-belleville/</t>
+  </si>
+  <si>
+    <t>Kirikou And The Sorceress</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/kirikou-and-the-sorceress/</t>
+  </si>
+  <si>
+    <t>Moonrise Kingdom</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/moonrise-kingdom/</t>
+  </si>
+  <si>
+    <t>Police Story</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/police-story/</t>
+  </si>
+  <si>
+    <t>Steamboat Bill Jr</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/steamboat-bill-jr/</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2296,6 +3205,14 @@
       <b/>
       <sz val="11"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -2330,16 +3247,19 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -2618,7 +3538,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D375"/>
+  <dimension ref="A1:D527"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="46.36328125" bestFit="1" customWidth="1"/>
@@ -6755,7 +7675,1692 @@
         <v>750</v>
       </c>
     </row>
+    <row r="376" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A376" t="s">
+        <v>751</v>
+      </c>
+      <c r="B376">
+        <v>1991</v>
+      </c>
+      <c r="D376" s="2" t="s">
+        <v>752</v>
+      </c>
+    </row>
+    <row r="377" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A377" t="s">
+        <v>753</v>
+      </c>
+      <c r="B377">
+        <v>2000</v>
+      </c>
+      <c r="D377" s="2" t="s">
+        <v>754</v>
+      </c>
+    </row>
+    <row r="378" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A378" t="s">
+        <v>755</v>
+      </c>
+      <c r="B378">
+        <v>1990</v>
+      </c>
+      <c r="D378" s="2" t="s">
+        <v>756</v>
+      </c>
+    </row>
+    <row r="379" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A379" t="s">
+        <v>757</v>
+      </c>
+      <c r="B379">
+        <v>1939</v>
+      </c>
+      <c r="D379" s="2" t="s">
+        <v>758</v>
+      </c>
+    </row>
+    <row r="380" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A380" t="s">
+        <v>759</v>
+      </c>
+      <c r="B380">
+        <v>1999</v>
+      </c>
+      <c r="D380" s="2" t="s">
+        <v>760</v>
+      </c>
+    </row>
+    <row r="381" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A381" t="s">
+        <v>761</v>
+      </c>
+      <c r="B381">
+        <v>2012</v>
+      </c>
+      <c r="D381" s="2" t="s">
+        <v>762</v>
+      </c>
+    </row>
+    <row r="382" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A382" t="s">
+        <v>763</v>
+      </c>
+      <c r="B382">
+        <v>1987</v>
+      </c>
+      <c r="D382" s="2" t="s">
+        <v>764</v>
+      </c>
+    </row>
+    <row r="383" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A383" t="s">
+        <v>765</v>
+      </c>
+      <c r="B383">
+        <v>1961</v>
+      </c>
+      <c r="D383" s="2" t="s">
+        <v>766</v>
+      </c>
+    </row>
+    <row r="384" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A384" t="s">
+        <v>767</v>
+      </c>
+      <c r="B384">
+        <v>2010</v>
+      </c>
+      <c r="D384" t="s">
+        <v>768</v>
+      </c>
+    </row>
+    <row r="385" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A385" t="s">
+        <v>769</v>
+      </c>
+      <c r="B385">
+        <v>1974</v>
+      </c>
+      <c r="D385" s="2" t="s">
+        <v>770</v>
+      </c>
+    </row>
+    <row r="386" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A386" t="s">
+        <v>771</v>
+      </c>
+      <c r="B386">
+        <v>1956</v>
+      </c>
+      <c r="D386" s="2" t="s">
+        <v>772</v>
+      </c>
+    </row>
+    <row r="387" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A387" t="s">
+        <v>773</v>
+      </c>
+      <c r="B387">
+        <v>2022</v>
+      </c>
+      <c r="D387" s="2" t="s">
+        <v>774</v>
+      </c>
+    </row>
+    <row r="388" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A388" t="s">
+        <v>775</v>
+      </c>
+      <c r="B388">
+        <v>2026</v>
+      </c>
+      <c r="D388" t="s">
+        <v>776</v>
+      </c>
+    </row>
+    <row r="389" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A389" t="s">
+        <v>777</v>
+      </c>
+      <c r="B389">
+        <v>1928</v>
+      </c>
+      <c r="D389" t="s">
+        <v>778</v>
+      </c>
+    </row>
+    <row r="390" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A390" t="s">
+        <v>779</v>
+      </c>
+      <c r="B390">
+        <v>1988</v>
+      </c>
+      <c r="D390" t="s">
+        <v>780</v>
+      </c>
+    </row>
+    <row r="391" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A391" t="s">
+        <v>781</v>
+      </c>
+      <c r="B391">
+        <v>1993</v>
+      </c>
+      <c r="D391" t="s">
+        <v>782</v>
+      </c>
+    </row>
+    <row r="392" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A392" t="s">
+        <v>783</v>
+      </c>
+      <c r="B392">
+        <v>1985</v>
+      </c>
+      <c r="D392" t="s">
+        <v>784</v>
+      </c>
+    </row>
+    <row r="393" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A393" t="s">
+        <v>785</v>
+      </c>
+      <c r="B393">
+        <v>1999</v>
+      </c>
+      <c r="D393" t="s">
+        <v>786</v>
+      </c>
+    </row>
+    <row r="394" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A394" t="s">
+        <v>787</v>
+      </c>
+      <c r="B394">
+        <v>1957</v>
+      </c>
+      <c r="D394" t="s">
+        <v>788</v>
+      </c>
+    </row>
+    <row r="395" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A395" t="s">
+        <v>789</v>
+      </c>
+      <c r="B395">
+        <v>2001</v>
+      </c>
+      <c r="D395" t="s">
+        <v>790</v>
+      </c>
+    </row>
+    <row r="396" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A396" t="s">
+        <v>791</v>
+      </c>
+      <c r="B396">
+        <v>1961</v>
+      </c>
+      <c r="D396" t="s">
+        <v>792</v>
+      </c>
+    </row>
+    <row r="397" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A397" t="s">
+        <v>793</v>
+      </c>
+      <c r="B397">
+        <v>2008</v>
+      </c>
+      <c r="D397" t="s">
+        <v>794</v>
+      </c>
+    </row>
+    <row r="398" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A398" t="s">
+        <v>795</v>
+      </c>
+      <c r="B398">
+        <v>2014</v>
+      </c>
+      <c r="D398" t="s">
+        <v>796</v>
+      </c>
+    </row>
+    <row r="399" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A399" t="s">
+        <v>797</v>
+      </c>
+      <c r="B399">
+        <v>1932</v>
+      </c>
+      <c r="D399" t="s">
+        <v>798</v>
+      </c>
+    </row>
+    <row r="400" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A400" t="s">
+        <v>799</v>
+      </c>
+      <c r="B400">
+        <v>2004</v>
+      </c>
+      <c r="D400" t="s">
+        <v>800</v>
+      </c>
+    </row>
+    <row r="401" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A401" t="s">
+        <v>801</v>
+      </c>
+      <c r="B401">
+        <v>2007</v>
+      </c>
+      <c r="D401" t="s">
+        <v>802</v>
+      </c>
+    </row>
+    <row r="402" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A402" t="s">
+        <v>803</v>
+      </c>
+      <c r="B402">
+        <v>1923</v>
+      </c>
+      <c r="D402" t="s">
+        <v>804</v>
+      </c>
+    </row>
+    <row r="403" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A403" t="s">
+        <v>805</v>
+      </c>
+      <c r="B403">
+        <v>1971</v>
+      </c>
+      <c r="D403" t="s">
+        <v>806</v>
+      </c>
+    </row>
+    <row r="404" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A404" t="s">
+        <v>807</v>
+      </c>
+      <c r="B404">
+        <v>1972</v>
+      </c>
+      <c r="D404" t="s">
+        <v>808</v>
+      </c>
+    </row>
+    <row r="405" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A405" t="s">
+        <v>809</v>
+      </c>
+      <c r="B405">
+        <v>1988</v>
+      </c>
+      <c r="D405" t="s">
+        <v>810</v>
+      </c>
+    </row>
+    <row r="406" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A406" t="s">
+        <v>811</v>
+      </c>
+      <c r="B406">
+        <v>1988</v>
+      </c>
+      <c r="D406" t="s">
+        <v>812</v>
+      </c>
+    </row>
+    <row r="407" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A407" t="s">
+        <v>813</v>
+      </c>
+      <c r="B407">
+        <v>1995</v>
+      </c>
+      <c r="D407" t="s">
+        <v>814</v>
+      </c>
+    </row>
+    <row r="408" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A408" t="s">
+        <v>815</v>
+      </c>
+      <c r="B408">
+        <v>1947</v>
+      </c>
+      <c r="D408" t="s">
+        <v>816</v>
+      </c>
+    </row>
+    <row r="409" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A409" t="s">
+        <v>817</v>
+      </c>
+      <c r="B409">
+        <v>1946</v>
+      </c>
+      <c r="D409" t="s">
+        <v>818</v>
+      </c>
+    </row>
+    <row r="410" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A410" t="s">
+        <v>819</v>
+      </c>
+      <c r="B410">
+        <v>1973</v>
+      </c>
+      <c r="D410" t="s">
+        <v>820</v>
+      </c>
+    </row>
+    <row r="411" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A411" t="s">
+        <v>821</v>
+      </c>
+      <c r="B411">
+        <v>1972</v>
+      </c>
+      <c r="D411" t="s">
+        <v>822</v>
+      </c>
+    </row>
+    <row r="412" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A412" t="s">
+        <v>823</v>
+      </c>
+      <c r="B412">
+        <v>1932</v>
+      </c>
+      <c r="D412" t="s">
+        <v>824</v>
+      </c>
+    </row>
+    <row r="413" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A413" t="s">
+        <v>825</v>
+      </c>
+      <c r="B413">
+        <v>1953</v>
+      </c>
+      <c r="D413" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="414" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A414" t="s">
+        <v>827</v>
+      </c>
+      <c r="B414">
+        <v>2004</v>
+      </c>
+      <c r="D414" t="s">
+        <v>828</v>
+      </c>
+    </row>
+    <row r="415" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A415" t="s">
+        <v>829</v>
+      </c>
+      <c r="B415">
+        <v>1961</v>
+      </c>
+      <c r="D415" t="s">
+        <v>830</v>
+      </c>
+    </row>
+    <row r="416" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A416" t="s">
+        <v>831</v>
+      </c>
+      <c r="B416">
+        <v>1991</v>
+      </c>
+      <c r="D416" t="s">
+        <v>832</v>
+      </c>
+    </row>
+    <row r="417" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A417" t="s">
+        <v>833</v>
+      </c>
+      <c r="B417">
+        <v>2009</v>
+      </c>
+      <c r="D417" t="s">
+        <v>834</v>
+      </c>
+    </row>
+    <row r="418" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A418" t="s">
+        <v>835</v>
+      </c>
+      <c r="B418">
+        <v>2013</v>
+      </c>
+      <c r="D418" t="s">
+        <v>836</v>
+      </c>
+    </row>
+    <row r="419" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A419" t="s">
+        <v>837</v>
+      </c>
+      <c r="B419">
+        <v>1986</v>
+      </c>
+      <c r="D419" t="s">
+        <v>838</v>
+      </c>
+    </row>
+    <row r="420" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A420" t="s">
+        <v>839</v>
+      </c>
+      <c r="B420">
+        <v>2021</v>
+      </c>
+      <c r="D420" t="s">
+        <v>840</v>
+      </c>
+    </row>
+    <row r="421" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A421" t="s">
+        <v>841</v>
+      </c>
+      <c r="B421">
+        <v>1958</v>
+      </c>
+      <c r="D421" t="s">
+        <v>842</v>
+      </c>
+    </row>
+    <row r="422" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A422" t="s">
+        <v>843</v>
+      </c>
+      <c r="B422">
+        <v>1987</v>
+      </c>
+      <c r="D422" t="s">
+        <v>844</v>
+      </c>
+    </row>
+    <row r="423" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A423" t="s">
+        <v>845</v>
+      </c>
+      <c r="B423">
+        <v>2006</v>
+      </c>
+      <c r="D423" t="s">
+        <v>846</v>
+      </c>
+    </row>
+    <row r="424" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A424" t="s">
+        <v>847</v>
+      </c>
+      <c r="B424">
+        <v>1985</v>
+      </c>
+      <c r="D424" t="s">
+        <v>848</v>
+      </c>
+    </row>
+    <row r="425" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A425" t="s">
+        <v>849</v>
+      </c>
+      <c r="B425">
+        <v>1961</v>
+      </c>
+      <c r="D425" t="s">
+        <v>850</v>
+      </c>
+    </row>
+    <row r="426" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A426" t="s">
+        <v>851</v>
+      </c>
+      <c r="B426">
+        <v>1978</v>
+      </c>
+      <c r="D426" t="s">
+        <v>852</v>
+      </c>
+    </row>
+    <row r="427" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A427" t="s">
+        <v>853</v>
+      </c>
+      <c r="B427">
+        <v>2011</v>
+      </c>
+      <c r="D427" t="s">
+        <v>854</v>
+      </c>
+    </row>
+    <row r="428" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A428" t="s">
+        <v>855</v>
+      </c>
+      <c r="B428">
+        <v>2016</v>
+      </c>
+      <c r="D428" t="s">
+        <v>856</v>
+      </c>
+    </row>
+    <row r="429" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A429" t="s">
+        <v>857</v>
+      </c>
+      <c r="B429">
+        <v>1995</v>
+      </c>
+      <c r="D429" t="s">
+        <v>858</v>
+      </c>
+    </row>
+    <row r="430" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A430" t="s">
+        <v>859</v>
+      </c>
+      <c r="B430">
+        <v>1928</v>
+      </c>
+      <c r="D430" t="s">
+        <v>860</v>
+      </c>
+    </row>
+    <row r="431" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A431" t="s">
+        <v>861</v>
+      </c>
+      <c r="B431">
+        <v>2022</v>
+      </c>
+      <c r="D431" t="s">
+        <v>862</v>
+      </c>
+    </row>
+    <row r="432" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A432" t="s">
+        <v>863</v>
+      </c>
+      <c r="B432">
+        <v>2017</v>
+      </c>
+      <c r="D432" t="s">
+        <v>864</v>
+      </c>
+    </row>
+    <row r="433" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A433" t="s">
+        <v>865</v>
+      </c>
+      <c r="B433">
+        <v>1980</v>
+      </c>
+      <c r="D433" t="s">
+        <v>866</v>
+      </c>
+    </row>
+    <row r="434" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A434" t="s">
+        <v>867</v>
+      </c>
+      <c r="B434">
+        <v>2024</v>
+      </c>
+      <c r="D434" t="s">
+        <v>868</v>
+      </c>
+    </row>
+    <row r="435" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A435" t="s">
+        <v>869</v>
+      </c>
+      <c r="B435">
+        <v>1948</v>
+      </c>
+      <c r="D435" t="s">
+        <v>870</v>
+      </c>
+    </row>
+    <row r="436" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A436" t="s">
+        <v>871</v>
+      </c>
+      <c r="B436">
+        <v>2011</v>
+      </c>
+      <c r="D436" t="s">
+        <v>872</v>
+      </c>
+    </row>
+    <row r="437" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A437" t="s">
+        <v>873</v>
+      </c>
+      <c r="B437">
+        <v>1952</v>
+      </c>
+      <c r="D437" t="s">
+        <v>874</v>
+      </c>
+    </row>
+    <row r="438" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A438" t="s">
+        <v>875</v>
+      </c>
+      <c r="B438">
+        <v>2025</v>
+      </c>
+      <c r="D438" t="s">
+        <v>876</v>
+      </c>
+    </row>
+    <row r="439" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A439" t="s">
+        <v>877</v>
+      </c>
+      <c r="B439">
+        <v>1950</v>
+      </c>
+      <c r="D439" t="s">
+        <v>878</v>
+      </c>
+    </row>
+    <row r="440" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A440" t="s">
+        <v>879</v>
+      </c>
+      <c r="B440">
+        <v>1966</v>
+      </c>
+      <c r="D440" t="s">
+        <v>880</v>
+      </c>
+    </row>
+    <row r="441" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A441" t="s">
+        <v>881</v>
+      </c>
+      <c r="B441">
+        <v>1964</v>
+      </c>
+      <c r="D441" t="s">
+        <v>882</v>
+      </c>
+    </row>
+    <row r="442" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A442" t="s">
+        <v>883</v>
+      </c>
+      <c r="B442">
+        <v>1946</v>
+      </c>
+      <c r="D442" t="s">
+        <v>884</v>
+      </c>
+    </row>
+    <row r="443" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A443" t="s">
+        <v>885</v>
+      </c>
+      <c r="B443">
+        <v>2018</v>
+      </c>
+      <c r="D443" t="s">
+        <v>886</v>
+      </c>
+    </row>
+    <row r="444" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A444" t="s">
+        <v>887</v>
+      </c>
+      <c r="B444">
+        <v>1960</v>
+      </c>
+      <c r="D444" t="s">
+        <v>888</v>
+      </c>
+    </row>
+    <row r="445" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A445" t="s">
+        <v>889</v>
+      </c>
+      <c r="B445">
+        <v>2001</v>
+      </c>
+      <c r="D445" t="s">
+        <v>890</v>
+      </c>
+    </row>
+    <row r="446" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A446" t="s">
+        <v>891</v>
+      </c>
+      <c r="B446">
+        <v>1966</v>
+      </c>
+      <c r="D446" t="s">
+        <v>892</v>
+      </c>
+    </row>
+    <row r="447" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A447" t="s">
+        <v>893</v>
+      </c>
+      <c r="B447">
+        <v>1986</v>
+      </c>
+      <c r="D447" t="s">
+        <v>894</v>
+      </c>
+    </row>
+    <row r="448" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A448" t="s">
+        <v>895</v>
+      </c>
+      <c r="B448">
+        <v>1966</v>
+      </c>
+      <c r="D448" t="s">
+        <v>896</v>
+      </c>
+    </row>
+    <row r="449" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A449" t="s">
+        <v>897</v>
+      </c>
+      <c r="B449">
+        <v>2001</v>
+      </c>
+      <c r="D449" t="s">
+        <v>898</v>
+      </c>
+    </row>
+    <row r="450" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A450" t="s">
+        <v>899</v>
+      </c>
+      <c r="B450">
+        <v>1999</v>
+      </c>
+      <c r="D450" t="s">
+        <v>900</v>
+      </c>
+    </row>
+    <row r="451" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A451" t="s">
+        <v>901</v>
+      </c>
+      <c r="B451">
+        <v>1997</v>
+      </c>
+      <c r="D451" t="s">
+        <v>902</v>
+      </c>
+    </row>
+    <row r="452" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A452" t="s">
+        <v>903</v>
+      </c>
+      <c r="B452">
+        <v>1998</v>
+      </c>
+      <c r="D452" t="s">
+        <v>904</v>
+      </c>
+    </row>
+    <row r="453" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A453" t="s">
+        <v>905</v>
+      </c>
+      <c r="B453">
+        <v>2017</v>
+      </c>
+      <c r="D453" t="s">
+        <v>906</v>
+      </c>
+    </row>
+    <row r="454" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A454" t="s">
+        <v>907</v>
+      </c>
+      <c r="B454">
+        <v>1946</v>
+      </c>
+      <c r="D454" t="s">
+        <v>908</v>
+      </c>
+    </row>
+    <row r="455" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A455" t="s">
+        <v>909</v>
+      </c>
+      <c r="B455">
+        <v>2005</v>
+      </c>
+      <c r="D455" t="s">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="456" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A456" t="s">
+        <v>911</v>
+      </c>
+      <c r="B456">
+        <v>1958</v>
+      </c>
+      <c r="D456" t="s">
+        <v>912</v>
+      </c>
+    </row>
+    <row r="457" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A457" t="s">
+        <v>913</v>
+      </c>
+      <c r="B457">
+        <v>1968</v>
+      </c>
+      <c r="D457" t="s">
+        <v>914</v>
+      </c>
+    </row>
+    <row r="458" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A458" t="s">
+        <v>915</v>
+      </c>
+      <c r="B458">
+        <v>2021</v>
+      </c>
+      <c r="D458" t="s">
+        <v>916</v>
+      </c>
+    </row>
+    <row r="459" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A459" t="s">
+        <v>917</v>
+      </c>
+      <c r="B459">
+        <v>2024</v>
+      </c>
+      <c r="D459" t="s">
+        <v>918</v>
+      </c>
+    </row>
+    <row r="460" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A460" t="s">
+        <v>919</v>
+      </c>
+      <c r="B460">
+        <v>1955</v>
+      </c>
+      <c r="D460" t="s">
+        <v>920</v>
+      </c>
+    </row>
+    <row r="461" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A461" t="s">
+        <v>921</v>
+      </c>
+      <c r="B461">
+        <v>1989</v>
+      </c>
+      <c r="D461" t="s">
+        <v>922</v>
+      </c>
+    </row>
+    <row r="462" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A462" t="s">
+        <v>923</v>
+      </c>
+      <c r="B462">
+        <v>2000</v>
+      </c>
+      <c r="D462" t="s">
+        <v>924</v>
+      </c>
+    </row>
+    <row r="463" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A463" t="s">
+        <v>925</v>
+      </c>
+      <c r="B463">
+        <v>1928</v>
+      </c>
+      <c r="D463" t="s">
+        <v>926</v>
+      </c>
+    </row>
+    <row r="464" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A464" t="s">
+        <v>927</v>
+      </c>
+      <c r="B464">
+        <v>2002</v>
+      </c>
+      <c r="D464" t="s">
+        <v>928</v>
+      </c>
+    </row>
+    <row r="465" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A465" t="s">
+        <v>929</v>
+      </c>
+      <c r="B465">
+        <v>1965</v>
+      </c>
+      <c r="D465" t="s">
+        <v>930</v>
+      </c>
+    </row>
+    <row r="466" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A466" t="s">
+        <v>931</v>
+      </c>
+      <c r="B466">
+        <v>2010</v>
+      </c>
+      <c r="D466" t="s">
+        <v>932</v>
+      </c>
+    </row>
+    <row r="467" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A467" t="s">
+        <v>933</v>
+      </c>
+      <c r="B467">
+        <v>2016</v>
+      </c>
+      <c r="D467" t="s">
+        <v>934</v>
+      </c>
+    </row>
+    <row r="468" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A468" t="s">
+        <v>935</v>
+      </c>
+      <c r="B468">
+        <v>1920</v>
+      </c>
+      <c r="D468" t="s">
+        <v>936</v>
+      </c>
+    </row>
+    <row r="469" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A469" t="s">
+        <v>937</v>
+      </c>
+      <c r="B469">
+        <v>1992</v>
+      </c>
+      <c r="D469" t="s">
+        <v>938</v>
+      </c>
+    </row>
+    <row r="470" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A470" t="s">
+        <v>939</v>
+      </c>
+      <c r="B470">
+        <v>1996</v>
+      </c>
+      <c r="D470" t="s">
+        <v>940</v>
+      </c>
+    </row>
+    <row r="471" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A471" t="s">
+        <v>941</v>
+      </c>
+      <c r="B471">
+        <v>1954</v>
+      </c>
+      <c r="D471" t="s">
+        <v>942</v>
+      </c>
+    </row>
+    <row r="472" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A472" t="s">
+        <v>943</v>
+      </c>
+      <c r="B472">
+        <v>2019</v>
+      </c>
+      <c r="D472" t="s">
+        <v>944</v>
+      </c>
+    </row>
+    <row r="473" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A473" t="s">
+        <v>945</v>
+      </c>
+      <c r="B473">
+        <v>1962</v>
+      </c>
+      <c r="D473" t="s">
+        <v>946</v>
+      </c>
+    </row>
+    <row r="474" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A474" t="s">
+        <v>947</v>
+      </c>
+      <c r="B474">
+        <v>2017</v>
+      </c>
+      <c r="D474" t="s">
+        <v>948</v>
+      </c>
+    </row>
+    <row r="475" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A475" t="s">
+        <v>949</v>
+      </c>
+      <c r="B475">
+        <v>1967</v>
+      </c>
+      <c r="D475" t="s">
+        <v>950</v>
+      </c>
+    </row>
+    <row r="476" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A476" t="s">
+        <v>951</v>
+      </c>
+      <c r="B476">
+        <v>1999</v>
+      </c>
+      <c r="D476" t="s">
+        <v>952</v>
+      </c>
+    </row>
+    <row r="477" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A477" t="s">
+        <v>953</v>
+      </c>
+      <c r="B477">
+        <v>1979</v>
+      </c>
+      <c r="D477" t="s">
+        <v>954</v>
+      </c>
+    </row>
+    <row r="478" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A478" t="s">
+        <v>955</v>
+      </c>
+      <c r="B478">
+        <v>1928</v>
+      </c>
+      <c r="D478" t="s">
+        <v>956</v>
+      </c>
+    </row>
+    <row r="479" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A479" t="s">
+        <v>957</v>
+      </c>
+      <c r="B479">
+        <v>1981</v>
+      </c>
+      <c r="D479" t="s">
+        <v>958</v>
+      </c>
+    </row>
+    <row r="480" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A480" t="s">
+        <v>959</v>
+      </c>
+      <c r="B480">
+        <v>1924</v>
+      </c>
+      <c r="D480" t="s">
+        <v>960</v>
+      </c>
+    </row>
+    <row r="481" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A481" t="s">
+        <v>961</v>
+      </c>
+      <c r="B481">
+        <v>2018</v>
+      </c>
+      <c r="D481" t="s">
+        <v>962</v>
+      </c>
+    </row>
+    <row r="482" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A482" t="s">
+        <v>963</v>
+      </c>
+      <c r="B482">
+        <v>1975</v>
+      </c>
+      <c r="D482" t="s">
+        <v>964</v>
+      </c>
+    </row>
+    <row r="483" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A483" t="s">
+        <v>965</v>
+      </c>
+      <c r="B483">
+        <v>2025</v>
+      </c>
+      <c r="D483" t="s">
+        <v>966</v>
+      </c>
+    </row>
+    <row r="484" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A484" t="s">
+        <v>967</v>
+      </c>
+      <c r="B484">
+        <v>1993</v>
+      </c>
+      <c r="D484" t="s">
+        <v>968</v>
+      </c>
+    </row>
+    <row r="485" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A485" t="s">
+        <v>969</v>
+      </c>
+      <c r="B485">
+        <v>1987</v>
+      </c>
+      <c r="D485" t="s">
+        <v>970</v>
+      </c>
+    </row>
+    <row r="486" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A486" t="s">
+        <v>971</v>
+      </c>
+      <c r="B486">
+        <v>1946</v>
+      </c>
+      <c r="D486" t="s">
+        <v>972</v>
+      </c>
+    </row>
+    <row r="487" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A487" t="s">
+        <v>973</v>
+      </c>
+      <c r="B487">
+        <v>2013</v>
+      </c>
+      <c r="D487" t="s">
+        <v>974</v>
+      </c>
+    </row>
+    <row r="488" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A488" t="s">
+        <v>975</v>
+      </c>
+      <c r="B488">
+        <v>1976</v>
+      </c>
+      <c r="D488" t="s">
+        <v>976</v>
+      </c>
+    </row>
+    <row r="489" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A489" t="s">
+        <v>977</v>
+      </c>
+      <c r="B489">
+        <v>2020</v>
+      </c>
+      <c r="D489" t="s">
+        <v>978</v>
+      </c>
+    </row>
+    <row r="490" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A490" t="s">
+        <v>979</v>
+      </c>
+      <c r="B490">
+        <v>1944</v>
+      </c>
+      <c r="D490" t="s">
+        <v>980</v>
+      </c>
+    </row>
+    <row r="491" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A491" t="s">
+        <v>981</v>
+      </c>
+      <c r="B491">
+        <v>2024</v>
+      </c>
+      <c r="D491" t="s">
+        <v>982</v>
+      </c>
+    </row>
+    <row r="492" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A492" t="s">
+        <v>983</v>
+      </c>
+      <c r="B492">
+        <v>1980</v>
+      </c>
+      <c r="D492" t="s">
+        <v>984</v>
+      </c>
+    </row>
+    <row r="493" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A493" t="s">
+        <v>985</v>
+      </c>
+      <c r="B493">
+        <v>1960</v>
+      </c>
+      <c r="D493" t="s">
+        <v>986</v>
+      </c>
+    </row>
+    <row r="494" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A494" t="s">
+        <v>987</v>
+      </c>
+      <c r="B494">
+        <v>2011</v>
+      </c>
+      <c r="D494" t="s">
+        <v>988</v>
+      </c>
+    </row>
+    <row r="495" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A495" t="s">
+        <v>989</v>
+      </c>
+      <c r="B495">
+        <v>1968</v>
+      </c>
+      <c r="D495" t="s">
+        <v>990</v>
+      </c>
+    </row>
+    <row r="496" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A496" t="s">
+        <v>991</v>
+      </c>
+      <c r="B496">
+        <v>2002</v>
+      </c>
+      <c r="D496" t="s">
+        <v>992</v>
+      </c>
+    </row>
+    <row r="497" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A497" t="s">
+        <v>993</v>
+      </c>
+      <c r="B497">
+        <v>2016</v>
+      </c>
+      <c r="D497" t="s">
+        <v>994</v>
+      </c>
+    </row>
+    <row r="498" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A498" t="s">
+        <v>995</v>
+      </c>
+      <c r="B498">
+        <v>2010</v>
+      </c>
+      <c r="D498" t="s">
+        <v>996</v>
+      </c>
+    </row>
+    <row r="499" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A499" t="s">
+        <v>997</v>
+      </c>
+      <c r="B499">
+        <v>1984</v>
+      </c>
+      <c r="D499" t="s">
+        <v>998</v>
+      </c>
+    </row>
+    <row r="500" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A500" t="s">
+        <v>999</v>
+      </c>
+      <c r="B500">
+        <v>1987</v>
+      </c>
+      <c r="D500" t="s">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="501" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A501" t="s">
+        <v>1001</v>
+      </c>
+      <c r="B501">
+        <v>1950</v>
+      </c>
+      <c r="D501" t="s">
+        <v>1002</v>
+      </c>
+    </row>
+    <row r="502" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A502" t="s">
+        <v>1003</v>
+      </c>
+      <c r="B502">
+        <v>1994</v>
+      </c>
+      <c r="D502" t="s">
+        <v>1004</v>
+      </c>
+    </row>
+    <row r="503" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A503" t="s">
+        <v>1005</v>
+      </c>
+      <c r="B503">
+        <v>2021</v>
+      </c>
+      <c r="D503" t="s">
+        <v>1006</v>
+      </c>
+    </row>
+    <row r="504" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A504" t="s">
+        <v>1007</v>
+      </c>
+      <c r="B504">
+        <v>2014</v>
+      </c>
+      <c r="D504" t="s">
+        <v>1008</v>
+      </c>
+    </row>
+    <row r="505" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A505" t="s">
+        <v>1009</v>
+      </c>
+      <c r="B505">
+        <v>1985</v>
+      </c>
+      <c r="D505" t="s">
+        <v>1010</v>
+      </c>
+    </row>
+    <row r="506" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A506" t="s">
+        <v>1011</v>
+      </c>
+      <c r="B506">
+        <v>1998</v>
+      </c>
+      <c r="D506" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="507" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A507" t="s">
+        <v>1013</v>
+      </c>
+      <c r="B507">
+        <v>2019</v>
+      </c>
+      <c r="D507" t="s">
+        <v>1014</v>
+      </c>
+    </row>
+    <row r="508" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A508" t="s">
+        <v>1015</v>
+      </c>
+      <c r="B508">
+        <v>2015</v>
+      </c>
+      <c r="D508" t="s">
+        <v>1016</v>
+      </c>
+    </row>
+    <row r="509" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A509" t="s">
+        <v>1017</v>
+      </c>
+      <c r="B509">
+        <v>2009</v>
+      </c>
+      <c r="D509" t="s">
+        <v>1018</v>
+      </c>
+    </row>
+    <row r="510" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A510" t="s">
+        <v>1019</v>
+      </c>
+      <c r="B510">
+        <v>2012</v>
+      </c>
+      <c r="D510" t="s">
+        <v>1020</v>
+      </c>
+    </row>
+    <row r="511" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A511" t="s">
+        <v>1021</v>
+      </c>
+      <c r="B511">
+        <v>1940</v>
+      </c>
+      <c r="D511" t="s">
+        <v>1022</v>
+      </c>
+    </row>
+    <row r="512" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A512" t="s">
+        <v>1023</v>
+      </c>
+      <c r="B512">
+        <v>2004</v>
+      </c>
+      <c r="D512" t="s">
+        <v>1024</v>
+      </c>
+    </row>
+    <row r="513" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A513" t="s">
+        <v>1025</v>
+      </c>
+      <c r="B513">
+        <v>1964</v>
+      </c>
+      <c r="D513" t="s">
+        <v>1026</v>
+      </c>
+    </row>
+    <row r="514" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A514" t="s">
+        <v>1027</v>
+      </c>
+      <c r="B514">
+        <v>2004</v>
+      </c>
+      <c r="D514" t="s">
+        <v>1028</v>
+      </c>
+    </row>
+    <row r="515" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A515" t="s">
+        <v>1029</v>
+      </c>
+      <c r="B515">
+        <v>2024</v>
+      </c>
+      <c r="D515" t="s">
+        <v>1030</v>
+      </c>
+    </row>
+    <row r="516" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A516" t="s">
+        <v>1031</v>
+      </c>
+      <c r="B516">
+        <v>1972</v>
+      </c>
+      <c r="D516" t="s">
+        <v>1032</v>
+      </c>
+    </row>
+    <row r="517" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A517" t="s">
+        <v>1033</v>
+      </c>
+      <c r="B517">
+        <v>1992</v>
+      </c>
+      <c r="D517" t="s">
+        <v>1034</v>
+      </c>
+    </row>
+    <row r="518" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A518" t="s">
+        <v>1035</v>
+      </c>
+      <c r="B518">
+        <v>2009</v>
+      </c>
+      <c r="D518" t="s">
+        <v>1036</v>
+      </c>
+    </row>
+    <row r="519" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A519" t="s">
+        <v>1037</v>
+      </c>
+      <c r="B519">
+        <v>1984</v>
+      </c>
+      <c r="D519" t="s">
+        <v>1038</v>
+      </c>
+    </row>
+    <row r="520" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A520" t="s">
+        <v>513</v>
+      </c>
+      <c r="B520">
+        <v>1980</v>
+      </c>
+      <c r="D520" t="s">
+        <v>1039</v>
+      </c>
+    </row>
+    <row r="521" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A521" t="s">
+        <v>1040</v>
+      </c>
+      <c r="B521">
+        <v>2003</v>
+      </c>
+      <c r="D521" t="s">
+        <v>1041</v>
+      </c>
+    </row>
+    <row r="522" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A522" t="s">
+        <v>1042</v>
+      </c>
+      <c r="B522">
+        <v>2008</v>
+      </c>
+      <c r="D522" t="s">
+        <v>1043</v>
+      </c>
+    </row>
+    <row r="523" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A523" t="s">
+        <v>1044</v>
+      </c>
+      <c r="B523">
+        <v>2003</v>
+      </c>
+      <c r="D523" t="s">
+        <v>1045</v>
+      </c>
+    </row>
+    <row r="524" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A524" t="s">
+        <v>1046</v>
+      </c>
+      <c r="B524">
+        <v>1998</v>
+      </c>
+      <c r="D524" t="s">
+        <v>1047</v>
+      </c>
+    </row>
+    <row r="525" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A525" t="s">
+        <v>1048</v>
+      </c>
+      <c r="B525">
+        <v>2012</v>
+      </c>
+      <c r="D525" t="s">
+        <v>1049</v>
+      </c>
+    </row>
+    <row r="526" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A526" t="s">
+        <v>1050</v>
+      </c>
+      <c r="B526">
+        <v>1985</v>
+      </c>
+      <c r="D526" t="s">
+        <v>1051</v>
+      </c>
+    </row>
+    <row r="527" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A527" t="s">
+        <v>1052</v>
+      </c>
+      <c r="B527">
+        <v>1928</v>
+      </c>
+      <c r="D527" t="s">
+        <v>1053</v>
+      </c>
+    </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="D376" r:id="rId1" xr:uid="{E845355F-2512-4FEA-8B22-7261DB0AEF68}"/>
+    <hyperlink ref="D377" r:id="rId2" xr:uid="{0BABEE8A-8F45-47E1-A57B-B9CD3AD6300A}"/>
+    <hyperlink ref="D378" r:id="rId3" xr:uid="{8C35DED6-55FB-4D0F-BC67-11555078D011}"/>
+    <hyperlink ref="D379" r:id="rId4" xr:uid="{6236F1CA-23A5-4253-A673-1D1AC489343F}"/>
+    <hyperlink ref="D380" r:id="rId5" xr:uid="{C86998E7-D40B-4095-B2C1-413E1E5982F6}"/>
+    <hyperlink ref="D381" r:id="rId6" xr:uid="{F938ED9A-6735-4A64-8558-B5829A874738}"/>
+    <hyperlink ref="D382" r:id="rId7" xr:uid="{4D495342-2395-4F7B-89F5-9893D9EC3A96}"/>
+    <hyperlink ref="D383" r:id="rId8" xr:uid="{0AF84B25-9FD2-451C-8DA3-4E0F17F12AC9}"/>
+    <hyperlink ref="D385" r:id="rId9" xr:uid="{776C9CEA-7871-4374-A43D-DFF17F3051B4}"/>
+    <hyperlink ref="D386" r:id="rId10" xr:uid="{454DB360-E518-429F-A862-554126EEE6A1}"/>
+    <hyperlink ref="D387" r:id="rId11" xr:uid="{368B7CDE-8355-4739-83B5-7B0ABB90B5B2}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Adding official stand up list
</commit_message>
<xml_diff>
--- a/Official Whitelist.xlsx
+++ b/Official Whitelist.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bigba\aa Personal Projects\Letterboxd-List-Scraping\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26ECD877-48C1-48D8-B674-4BD61141BA05}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29E26AEC-88BC-4C3F-BA75-6A91EA408255}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1101" uniqueCount="1100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1109" uniqueCount="1108">
   <si>
     <t>Title</t>
   </si>
@@ -3060,12 +3060,6 @@
     <t>https://letterboxd.com/film/buddies-1985/</t>
   </si>
   <si>
-    <t>The Boys</t>
-  </si>
-  <si>
-    <t>https://letterboxd.com/film/the-boys/</t>
-  </si>
-  <si>
     <t>Maronas Fantastic Tale</t>
   </si>
   <si>
@@ -3325,6 +3319,36 @@
   </si>
   <si>
     <t>https://letterboxd.com/film/pelle-the-conqueror/</t>
+  </si>
+  <si>
+    <t>Haikyu The Dumpster Battle</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/haikyu-the-dumpster-battle/</t>
+  </si>
+  <si>
+    <t>The Runner</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/the-runner/</t>
+  </si>
+  <si>
+    <t>Barbie Princess Charm School</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/barbie-princess-charm-school/</t>
+  </si>
+  <si>
+    <t>Scenes From A Marriage</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/scenes-from-a-marriage/</t>
+  </si>
+  <si>
+    <t>C O Kancharapalem</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/c-o-kancharapalem/</t>
   </si>
 </sst>
 </file>
@@ -3676,7 +3700,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D550"/>
+  <dimension ref="A1:D554"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="46.36328125" bestFit="1" customWidth="1"/>
@@ -9248,7 +9272,7 @@
         <v>1011</v>
       </c>
       <c r="B506">
-        <v>1998</v>
+        <v>2019</v>
       </c>
       <c r="D506" t="s">
         <v>1012</v>
@@ -9259,7 +9283,7 @@
         <v>1013</v>
       </c>
       <c r="B507">
-        <v>2019</v>
+        <v>2015</v>
       </c>
       <c r="D507" t="s">
         <v>1014</v>
@@ -9270,7 +9294,7 @@
         <v>1015</v>
       </c>
       <c r="B508">
-        <v>2015</v>
+        <v>2009</v>
       </c>
       <c r="D508" t="s">
         <v>1016</v>
@@ -9281,7 +9305,7 @@
         <v>1017</v>
       </c>
       <c r="B509">
-        <v>2009</v>
+        <v>2012</v>
       </c>
       <c r="D509" t="s">
         <v>1018</v>
@@ -9292,7 +9316,7 @@
         <v>1019</v>
       </c>
       <c r="B510">
-        <v>2012</v>
+        <v>1940</v>
       </c>
       <c r="D510" t="s">
         <v>1020</v>
@@ -9303,7 +9327,7 @@
         <v>1021</v>
       </c>
       <c r="B511">
-        <v>1940</v>
+        <v>2004</v>
       </c>
       <c r="D511" t="s">
         <v>1022</v>
@@ -9314,7 +9338,7 @@
         <v>1023</v>
       </c>
       <c r="B512">
-        <v>2004</v>
+        <v>1964</v>
       </c>
       <c r="D512" t="s">
         <v>1024</v>
@@ -9325,7 +9349,7 @@
         <v>1025</v>
       </c>
       <c r="B513">
-        <v>1964</v>
+        <v>2004</v>
       </c>
       <c r="D513" t="s">
         <v>1026</v>
@@ -9336,7 +9360,7 @@
         <v>1027</v>
       </c>
       <c r="B514">
-        <v>2004</v>
+        <v>2024</v>
       </c>
       <c r="D514" t="s">
         <v>1028</v>
@@ -9347,7 +9371,7 @@
         <v>1029</v>
       </c>
       <c r="B515">
-        <v>2024</v>
+        <v>1972</v>
       </c>
       <c r="D515" t="s">
         <v>1030</v>
@@ -9358,7 +9382,7 @@
         <v>1031</v>
       </c>
       <c r="B516">
-        <v>1972</v>
+        <v>1992</v>
       </c>
       <c r="D516" t="s">
         <v>1032</v>
@@ -9369,7 +9393,7 @@
         <v>1033</v>
       </c>
       <c r="B517">
-        <v>1992</v>
+        <v>2009</v>
       </c>
       <c r="D517" t="s">
         <v>1034</v>
@@ -9380,7 +9404,7 @@
         <v>1035</v>
       </c>
       <c r="B518">
-        <v>2009</v>
+        <v>1984</v>
       </c>
       <c r="D518" t="s">
         <v>1036</v>
@@ -9388,21 +9412,21 @@
     </row>
     <row r="519" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A519" t="s">
+        <v>513</v>
+      </c>
+      <c r="B519">
+        <v>1980</v>
+      </c>
+      <c r="D519" t="s">
         <v>1037</v>
-      </c>
-      <c r="B519">
-        <v>1984</v>
-      </c>
-      <c r="D519" t="s">
-        <v>1038</v>
       </c>
     </row>
     <row r="520" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A520" t="s">
-        <v>513</v>
+        <v>1038</v>
       </c>
       <c r="B520">
-        <v>1980</v>
+        <v>2003</v>
       </c>
       <c r="D520" t="s">
         <v>1039</v>
@@ -9413,7 +9437,7 @@
         <v>1040</v>
       </c>
       <c r="B521">
-        <v>2003</v>
+        <v>2008</v>
       </c>
       <c r="D521" t="s">
         <v>1041</v>
@@ -9424,7 +9448,7 @@
         <v>1042</v>
       </c>
       <c r="B522">
-        <v>2008</v>
+        <v>2003</v>
       </c>
       <c r="D522" t="s">
         <v>1043</v>
@@ -9435,7 +9459,7 @@
         <v>1044</v>
       </c>
       <c r="B523">
-        <v>2003</v>
+        <v>1998</v>
       </c>
       <c r="D523" t="s">
         <v>1045</v>
@@ -9446,7 +9470,7 @@
         <v>1046</v>
       </c>
       <c r="B524">
-        <v>1998</v>
+        <v>2012</v>
       </c>
       <c r="D524" t="s">
         <v>1047</v>
@@ -9457,7 +9481,7 @@
         <v>1048</v>
       </c>
       <c r="B525">
-        <v>2012</v>
+        <v>1985</v>
       </c>
       <c r="D525" t="s">
         <v>1049</v>
@@ -9468,7 +9492,7 @@
         <v>1050</v>
       </c>
       <c r="B526">
-        <v>1985</v>
+        <v>1928</v>
       </c>
       <c r="D526" t="s">
         <v>1051</v>
@@ -9479,9 +9503,9 @@
         <v>1052</v>
       </c>
       <c r="B527">
-        <v>1928</v>
-      </c>
-      <c r="D527" t="s">
+        <v>1969</v>
+      </c>
+      <c r="D527" s="2" t="s">
         <v>1053</v>
       </c>
     </row>
@@ -9490,9 +9514,9 @@
         <v>1054</v>
       </c>
       <c r="B528">
-        <v>1969</v>
-      </c>
-      <c r="D528" s="2" t="s">
+        <v>1982</v>
+      </c>
+      <c r="D528" t="s">
         <v>1055</v>
       </c>
     </row>
@@ -9501,7 +9525,7 @@
         <v>1056</v>
       </c>
       <c r="B529">
-        <v>1982</v>
+        <v>1948</v>
       </c>
       <c r="D529" t="s">
         <v>1057</v>
@@ -9512,7 +9536,7 @@
         <v>1058</v>
       </c>
       <c r="B530">
-        <v>1948</v>
+        <v>1968</v>
       </c>
       <c r="D530" t="s">
         <v>1059</v>
@@ -9523,7 +9547,7 @@
         <v>1060</v>
       </c>
       <c r="B531">
-        <v>1968</v>
+        <v>1971</v>
       </c>
       <c r="D531" t="s">
         <v>1061</v>
@@ -9534,7 +9558,7 @@
         <v>1062</v>
       </c>
       <c r="B532">
-        <v>1971</v>
+        <v>2025</v>
       </c>
       <c r="D532" t="s">
         <v>1063</v>
@@ -9545,7 +9569,7 @@
         <v>1064</v>
       </c>
       <c r="B533">
-        <v>2025</v>
+        <v>2004</v>
       </c>
       <c r="D533" t="s">
         <v>1065</v>
@@ -9556,7 +9580,7 @@
         <v>1066</v>
       </c>
       <c r="B534">
-        <v>2004</v>
+        <v>2025</v>
       </c>
       <c r="D534" t="s">
         <v>1067</v>
@@ -9567,7 +9591,7 @@
         <v>1068</v>
       </c>
       <c r="B535">
-        <v>2025</v>
+        <v>1992</v>
       </c>
       <c r="D535" t="s">
         <v>1069</v>
@@ -9578,7 +9602,7 @@
         <v>1070</v>
       </c>
       <c r="B536">
-        <v>1992</v>
+        <v>1990</v>
       </c>
       <c r="D536" t="s">
         <v>1071</v>
@@ -9589,7 +9613,7 @@
         <v>1072</v>
       </c>
       <c r="B537">
-        <v>1990</v>
+        <v>1949</v>
       </c>
       <c r="D537" t="s">
         <v>1073</v>
@@ -9600,7 +9624,7 @@
         <v>1074</v>
       </c>
       <c r="B538">
-        <v>1949</v>
+        <v>2023</v>
       </c>
       <c r="D538" t="s">
         <v>1075</v>
@@ -9611,7 +9635,7 @@
         <v>1076</v>
       </c>
       <c r="B539">
-        <v>2023</v>
+        <v>1964</v>
       </c>
       <c r="D539" t="s">
         <v>1077</v>
@@ -9622,7 +9646,7 @@
         <v>1078</v>
       </c>
       <c r="B540">
-        <v>1964</v>
+        <v>1986</v>
       </c>
       <c r="D540" t="s">
         <v>1079</v>
@@ -9633,7 +9657,7 @@
         <v>1080</v>
       </c>
       <c r="B541">
-        <v>1986</v>
+        <v>1977</v>
       </c>
       <c r="D541" t="s">
         <v>1081</v>
@@ -9644,7 +9668,7 @@
         <v>1082</v>
       </c>
       <c r="B542">
-        <v>1977</v>
+        <v>1972</v>
       </c>
       <c r="D542" t="s">
         <v>1083</v>
@@ -9655,7 +9679,7 @@
         <v>1084</v>
       </c>
       <c r="B543">
-        <v>1972</v>
+        <v>2000</v>
       </c>
       <c r="D543" t="s">
         <v>1085</v>
@@ -9666,7 +9690,7 @@
         <v>1086</v>
       </c>
       <c r="B544">
-        <v>2000</v>
+        <v>1994</v>
       </c>
       <c r="D544" t="s">
         <v>1087</v>
@@ -9677,7 +9701,7 @@
         <v>1088</v>
       </c>
       <c r="B545">
-        <v>1994</v>
+        <v>1990</v>
       </c>
       <c r="D545" t="s">
         <v>1089</v>
@@ -9688,7 +9712,7 @@
         <v>1090</v>
       </c>
       <c r="B546">
-        <v>1990</v>
+        <v>1999</v>
       </c>
       <c r="D546" t="s">
         <v>1091</v>
@@ -9699,7 +9723,7 @@
         <v>1092</v>
       </c>
       <c r="B547">
-        <v>1999</v>
+        <v>2011</v>
       </c>
       <c r="D547" t="s">
         <v>1093</v>
@@ -9710,7 +9734,7 @@
         <v>1094</v>
       </c>
       <c r="B548">
-        <v>2011</v>
+        <v>2004</v>
       </c>
       <c r="D548" t="s">
         <v>1095</v>
@@ -9721,7 +9745,7 @@
         <v>1096</v>
       </c>
       <c r="B549">
-        <v>2004</v>
+        <v>1987</v>
       </c>
       <c r="D549" t="s">
         <v>1097</v>
@@ -9732,10 +9756,54 @@
         <v>1098</v>
       </c>
       <c r="B550">
-        <v>1987</v>
+        <v>2024</v>
       </c>
       <c r="D550" t="s">
         <v>1099</v>
+      </c>
+    </row>
+    <row r="551" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A551" t="s">
+        <v>1100</v>
+      </c>
+      <c r="B551">
+        <v>1984</v>
+      </c>
+      <c r="D551" s="2" t="s">
+        <v>1101</v>
+      </c>
+    </row>
+    <row r="552" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A552" t="s">
+        <v>1102</v>
+      </c>
+      <c r="B552">
+        <v>2011</v>
+      </c>
+      <c r="D552" s="2" t="s">
+        <v>1103</v>
+      </c>
+    </row>
+    <row r="553" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A553" t="s">
+        <v>1104</v>
+      </c>
+      <c r="B553">
+        <v>1974</v>
+      </c>
+      <c r="D553" t="s">
+        <v>1105</v>
+      </c>
+    </row>
+    <row r="554" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A554" t="s">
+        <v>1106</v>
+      </c>
+      <c r="B554">
+        <v>2018</v>
+      </c>
+      <c r="D554" s="2" t="s">
+        <v>1107</v>
       </c>
     </row>
   </sheetData>
@@ -9751,7 +9819,10 @@
     <hyperlink ref="D385" r:id="rId9" xr:uid="{776C9CEA-7871-4374-A43D-DFF17F3051B4}"/>
     <hyperlink ref="D386" r:id="rId10" xr:uid="{454DB360-E518-429F-A862-554126EEE6A1}"/>
     <hyperlink ref="D387" r:id="rId11" xr:uid="{368B7CDE-8355-4739-83B5-7B0ABB90B5B2}"/>
-    <hyperlink ref="D528" r:id="rId12" xr:uid="{A4301CC4-9A54-49C3-8360-6DD0E8DCE230}"/>
+    <hyperlink ref="D527" r:id="rId12" xr:uid="{A4301CC4-9A54-49C3-8360-6DD0E8DCE230}"/>
+    <hyperlink ref="D551" r:id="rId13" xr:uid="{16145F1C-6214-4749-8D8A-FDD477E08B28}"/>
+    <hyperlink ref="D552" r:id="rId14" xr:uid="{024C5F8B-8F81-420D-868D-5D8E76ABB1AE}"/>
+    <hyperlink ref="D554" r:id="rId15" xr:uid="{E70978B9-40E5-446D-987D-E57F6DB2DA9E}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Various tweaks. new official comedy list.
</commit_message>
<xml_diff>
--- a/Official Whitelist.xlsx
+++ b/Official Whitelist.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bigba\aa Personal Projects\Letterboxd-List-Scraping\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29E26AEC-88BC-4C3F-BA75-6A91EA408255}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{286A05FB-9B42-4F3E-A79D-97E51079085E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1109" uniqueCount="1108">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1120" uniqueCount="1119">
   <si>
     <t>Title</t>
   </si>
@@ -3349,6 +3349,39 @@
   </si>
   <si>
     <t>https://letterboxd.com/film/c-o-kancharapalem/</t>
+  </si>
+  <si>
+    <t>Stormskerry Maja</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/stormskerry-maja/</t>
+  </si>
+  <si>
+    <t>Time Still Turns The Pages</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/time-still-turns-the-pages/</t>
+  </si>
+  <si>
+    <t>Yes</t>
+  </si>
+  <si>
+    <t>Walking the Streets of Moscow</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/walking-the-streets-of-moscow/</t>
+  </si>
+  <si>
+    <t>War And Peace Part Ii Natasha Rostova</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/war-and-peace-part-ii-natasha-rostova/</t>
+  </si>
+  <si>
+    <t>Castration Movie Anthology i. Traps</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/castration-movie-anthology-i-traps/</t>
   </si>
 </sst>
 </file>
@@ -3700,7 +3733,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D554"/>
+  <dimension ref="A1:E559"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="46.36328125" bestFit="1" customWidth="1"/>
@@ -9696,7 +9729,7 @@
         <v>1087</v>
       </c>
     </row>
-    <row r="545" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="545" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A545" t="s">
         <v>1088</v>
       </c>
@@ -9707,7 +9740,7 @@
         <v>1089</v>
       </c>
     </row>
-    <row r="546" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="546" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A546" t="s">
         <v>1090</v>
       </c>
@@ -9718,7 +9751,7 @@
         <v>1091</v>
       </c>
     </row>
-    <row r="547" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="547" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A547" t="s">
         <v>1092</v>
       </c>
@@ -9729,7 +9762,7 @@
         <v>1093</v>
       </c>
     </row>
-    <row r="548" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="548" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A548" t="s">
         <v>1094</v>
       </c>
@@ -9740,7 +9773,7 @@
         <v>1095</v>
       </c>
     </row>
-    <row r="549" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="549" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A549" t="s">
         <v>1096</v>
       </c>
@@ -9751,7 +9784,7 @@
         <v>1097</v>
       </c>
     </row>
-    <row r="550" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="550" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A550" t="s">
         <v>1098</v>
       </c>
@@ -9762,7 +9795,7 @@
         <v>1099</v>
       </c>
     </row>
-    <row r="551" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="551" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A551" t="s">
         <v>1100</v>
       </c>
@@ -9773,7 +9806,7 @@
         <v>1101</v>
       </c>
     </row>
-    <row r="552" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="552" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A552" t="s">
         <v>1102</v>
       </c>
@@ -9784,7 +9817,7 @@
         <v>1103</v>
       </c>
     </row>
-    <row r="553" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="553" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A553" t="s">
         <v>1104</v>
       </c>
@@ -9795,7 +9828,7 @@
         <v>1105</v>
       </c>
     </row>
-    <row r="554" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="554" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A554" t="s">
         <v>1106</v>
       </c>
@@ -9804,6 +9837,79 @@
       </c>
       <c r="D554" s="2" t="s">
         <v>1107</v>
+      </c>
+    </row>
+    <row r="555" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A555" t="s">
+        <v>1108</v>
+      </c>
+      <c r="B555">
+        <v>2024</v>
+      </c>
+      <c r="C555">
+        <v>1028769</v>
+      </c>
+      <c r="D555" s="2" t="s">
+        <v>1109</v>
+      </c>
+    </row>
+    <row r="556" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A556" t="s">
+        <v>1110</v>
+      </c>
+      <c r="B556">
+        <v>2023</v>
+      </c>
+      <c r="C556">
+        <v>957863</v>
+      </c>
+      <c r="D556" s="2" t="s">
+        <v>1111</v>
+      </c>
+    </row>
+    <row r="557" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A557" t="s">
+        <v>1113</v>
+      </c>
+      <c r="B557">
+        <v>1964</v>
+      </c>
+      <c r="C557">
+        <v>27862</v>
+      </c>
+      <c r="D557" s="2" t="s">
+        <v>1114</v>
+      </c>
+    </row>
+    <row r="558" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A558" t="s">
+        <v>1115</v>
+      </c>
+      <c r="B558">
+        <v>1965</v>
+      </c>
+      <c r="C558">
+        <v>149465</v>
+      </c>
+      <c r="D558" s="2" t="s">
+        <v>1116</v>
+      </c>
+    </row>
+    <row r="559" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A559" t="s">
+        <v>1117</v>
+      </c>
+      <c r="B559">
+        <v>2024</v>
+      </c>
+      <c r="C559">
+        <v>1243479</v>
+      </c>
+      <c r="D559" s="2" t="s">
+        <v>1118</v>
+      </c>
+      <c r="E559" t="s">
+        <v>1112</v>
       </c>
     </row>
   </sheetData>
@@ -9823,6 +9929,11 @@
     <hyperlink ref="D551" r:id="rId13" xr:uid="{16145F1C-6214-4749-8D8A-FDD477E08B28}"/>
     <hyperlink ref="D552" r:id="rId14" xr:uid="{024C5F8B-8F81-420D-868D-5D8E76ABB1AE}"/>
     <hyperlink ref="D554" r:id="rId15" xr:uid="{E70978B9-40E5-446D-987D-E57F6DB2DA9E}"/>
+    <hyperlink ref="D555" r:id="rId16" xr:uid="{A294FD8A-3D0D-4D2E-87BD-F10BABD32315}"/>
+    <hyperlink ref="D556" r:id="rId17" xr:uid="{F28C7628-2B4D-4FCE-8952-BFDD7C7F06CE}"/>
+    <hyperlink ref="D557" r:id="rId18" xr:uid="{193BDB09-EFD2-4937-8E49-91638F1A9791}"/>
+    <hyperlink ref="D558" r:id="rId19" xr:uid="{5C1D518D-E5D1-4FFF-A746-E8BAD67AEA01}"/>
+    <hyperlink ref="D559" r:id="rId20" xr:uid="{5D8CCB0C-6663-42F7-A44C-954C049BD83E}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Updated nc-17 Rated list to be top 15
</commit_message>
<xml_diff>
--- a/Official Whitelist.xlsx
+++ b/Official Whitelist.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bigba\aa Personal Projects\Letterboxd-List-Scraping\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{12A0C7A8-C99F-4BAC-8F50-4194F13886C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{665A4384-62DC-4175-A287-E30D3F6DE382}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2080" yWindow="2080" windowWidth="14400" windowHeight="8170" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1138" uniqueCount="1135">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1137" uniqueCount="1136">
   <si>
     <t>Title</t>
   </si>
@@ -3363,9 +3363,6 @@
     <t>https://letterboxd.com/film/time-still-turns-the-pages/</t>
   </si>
   <si>
-    <t>Yes</t>
-  </si>
-  <si>
     <t>Walking the Streets of Moscow</t>
   </si>
   <si>
@@ -3430,6 +3427,12 @@
   </si>
   <si>
     <t>https://letterboxd.com/film/eros-massacre/</t>
+  </si>
+  <si>
+    <t>Sairat</t>
+  </si>
+  <si>
+    <t>https://letterboxd.com/film/sairat/</t>
   </si>
 </sst>
 </file>
@@ -3781,7 +3784,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E567"/>
+  <dimension ref="A1:D568"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="46.36328125" bestFit="1" customWidth="1"/>
@@ -9777,7 +9780,7 @@
         <v>1087</v>
       </c>
     </row>
-    <row r="545" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="545" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A545" t="s">
         <v>1088</v>
       </c>
@@ -9788,7 +9791,7 @@
         <v>1089</v>
       </c>
     </row>
-    <row r="546" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="546" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A546" t="s">
         <v>1090</v>
       </c>
@@ -9799,7 +9802,7 @@
         <v>1091</v>
       </c>
     </row>
-    <row r="547" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="547" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A547" t="s">
         <v>1092</v>
       </c>
@@ -9810,7 +9813,7 @@
         <v>1093</v>
       </c>
     </row>
-    <row r="548" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="548" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A548" t="s">
         <v>1094</v>
       </c>
@@ -9821,7 +9824,7 @@
         <v>1095</v>
       </c>
     </row>
-    <row r="549" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="549" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A549" t="s">
         <v>1096</v>
       </c>
@@ -9832,7 +9835,7 @@
         <v>1097</v>
       </c>
     </row>
-    <row r="550" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="550" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A550" t="s">
         <v>1098</v>
       </c>
@@ -9843,7 +9846,7 @@
         <v>1099</v>
       </c>
     </row>
-    <row r="551" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="551" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A551" t="s">
         <v>1100</v>
       </c>
@@ -9854,7 +9857,7 @@
         <v>1101</v>
       </c>
     </row>
-    <row r="552" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="552" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A552" t="s">
         <v>1102</v>
       </c>
@@ -9865,7 +9868,7 @@
         <v>1103</v>
       </c>
     </row>
-    <row r="553" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="553" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A553" t="s">
         <v>1104</v>
       </c>
@@ -9876,7 +9879,7 @@
         <v>1105</v>
       </c>
     </row>
-    <row r="554" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="554" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A554" t="s">
         <v>1106</v>
       </c>
@@ -9887,7 +9890,7 @@
         <v>1107</v>
       </c>
     </row>
-    <row r="555" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="555" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A555" t="s">
         <v>1108</v>
       </c>
@@ -9901,7 +9904,7 @@
         <v>1109</v>
       </c>
     </row>
-    <row r="556" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="556" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A556" t="s">
         <v>1110</v>
       </c>
@@ -9915,9 +9918,9 @@
         <v>1111</v>
       </c>
     </row>
-    <row r="557" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="557" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A557" t="s">
-        <v>1113</v>
+        <v>1112</v>
       </c>
       <c r="B557">
         <v>1964</v>
@@ -9926,12 +9929,12 @@
         <v>27862</v>
       </c>
       <c r="D557" s="2" t="s">
+        <v>1113</v>
+      </c>
+    </row>
+    <row r="558" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A558" t="s">
         <v>1114</v>
-      </c>
-    </row>
-    <row r="558" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A558" t="s">
-        <v>1115</v>
       </c>
       <c r="B558">
         <v>1965</v>
@@ -9940,12 +9943,12 @@
         <v>149465</v>
       </c>
       <c r="D558" s="2" t="s">
+        <v>1115</v>
+      </c>
+    </row>
+    <row r="559" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A559" t="s">
         <v>1116</v>
-      </c>
-    </row>
-    <row r="559" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A559" t="s">
-        <v>1117</v>
       </c>
       <c r="B559">
         <v>2024</v>
@@ -9954,15 +9957,12 @@
         <v>1243479</v>
       </c>
       <c r="D559" s="2" t="s">
+        <v>1117</v>
+      </c>
+    </row>
+    <row r="560" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A560" t="s">
         <v>1118</v>
-      </c>
-      <c r="E559" t="s">
-        <v>1112</v>
-      </c>
-    </row>
-    <row r="560" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A560" t="s">
-        <v>1119</v>
       </c>
       <c r="B560">
         <v>1984</v>
@@ -9971,15 +9971,12 @@
         <v>81</v>
       </c>
       <c r="D560" s="2" t="s">
+        <v>1119</v>
+      </c>
+    </row>
+    <row r="561" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A561" t="s">
         <v>1120</v>
-      </c>
-      <c r="E560" t="s">
-        <v>1112</v>
-      </c>
-    </row>
-    <row r="561" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A561" t="s">
-        <v>1121</v>
       </c>
       <c r="B561">
         <v>2008</v>
@@ -9988,15 +9985,12 @@
         <v>111188</v>
       </c>
       <c r="D561" s="2" t="s">
+        <v>1121</v>
+      </c>
+    </row>
+    <row r="562" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A562" t="s">
         <v>1122</v>
-      </c>
-      <c r="E561" t="s">
-        <v>1112</v>
-      </c>
-    </row>
-    <row r="562" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A562" t="s">
-        <v>1123</v>
       </c>
       <c r="B562">
         <v>1975</v>
@@ -10005,12 +9999,12 @@
         <v>511</v>
       </c>
       <c r="D562" s="2" t="s">
+        <v>1123</v>
+      </c>
+    </row>
+    <row r="563" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A563" t="s">
         <v>1124</v>
-      </c>
-    </row>
-    <row r="563" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A563" t="s">
-        <v>1125</v>
       </c>
       <c r="B563">
         <v>1992</v>
@@ -10019,12 +10013,12 @@
         <v>66362</v>
       </c>
       <c r="D563" s="2" t="s">
+        <v>1125</v>
+      </c>
+    </row>
+    <row r="564" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A564" t="s">
         <v>1126</v>
-      </c>
-    </row>
-    <row r="564" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A564" t="s">
-        <v>1127</v>
       </c>
       <c r="B564">
         <v>1989</v>
@@ -10033,12 +10027,12 @@
         <v>237957</v>
       </c>
       <c r="D564" t="s">
+        <v>1127</v>
+      </c>
+    </row>
+    <row r="565" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A565" t="s">
         <v>1128</v>
-      </c>
-    </row>
-    <row r="565" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A565" t="s">
-        <v>1129</v>
       </c>
       <c r="B565">
         <v>2004</v>
@@ -10047,12 +10041,12 @@
         <v>9470</v>
       </c>
       <c r="D565" s="2" t="s">
+        <v>1129</v>
+      </c>
+    </row>
+    <row r="566" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A566" t="s">
         <v>1130</v>
-      </c>
-    </row>
-    <row r="566" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A566" t="s">
-        <v>1131</v>
       </c>
       <c r="B566">
         <v>1987</v>
@@ -10061,12 +10055,12 @@
         <v>275366</v>
       </c>
       <c r="D566" t="s">
+        <v>1131</v>
+      </c>
+    </row>
+    <row r="567" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A567" t="s">
         <v>1132</v>
-      </c>
-    </row>
-    <row r="567" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A567" t="s">
-        <v>1133</v>
       </c>
       <c r="B567">
         <v>1969</v>
@@ -10075,7 +10069,21 @@
         <v>78117</v>
       </c>
       <c r="D567" t="s">
+        <v>1133</v>
+      </c>
+    </row>
+    <row r="568" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A568" t="s">
         <v>1134</v>
+      </c>
+      <c r="B568">
+        <v>2016</v>
+      </c>
+      <c r="C568">
+        <v>383367</v>
+      </c>
+      <c r="D568" s="2" t="s">
+        <v>1135</v>
       </c>
     </row>
   </sheetData>
@@ -10105,6 +10113,7 @@
     <hyperlink ref="D562" r:id="rId23" xr:uid="{B0DAA382-D612-4C52-92CC-60F966246E5A}"/>
     <hyperlink ref="D563" r:id="rId24" xr:uid="{F1F98DA8-9B33-4768-A093-3D35DBF11836}"/>
     <hyperlink ref="D565" r:id="rId25" xr:uid="{183D0A7D-6CE1-42F6-B6E1-4F9B48010CF2}"/>
+    <hyperlink ref="D568" r:id="rId26" xr:uid="{82067776-FBC4-42EE-8A1C-DC7F82929CE6}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>